<commit_message>
Protect the working column with an optional password
Testing what the protection actually buys: unhiding the hidden calculation
column is blocked, and locked cells cannot be selected, so a formula cannot be
read by clicking one. But Review > Unprotect Sheet was a single click, because
the sheets carried no password.

build_workbook.py --password closes that. Inputs are unlocked, so nobody typing
a deal is ever prompted - the brief's 'no password prompt' requirement still
holds; the password only guards the Unprotect button.

It remains a deterrent. An .xlsx is a zip and sheet protection is one XML
element inside it; stripping it removed protection from all three sheets in a
single pass, password or not. Documented rather than glossed over, because it
decides what can honestly be promised.

verify.py now passes the password explicitly - Unprotect() without one raises a
modal dialog that hangs headless Excel with no window to dismiss.
</commit_message>
<xml_diff>
--- a/output/property_feasibility.xlsx
+++ b/output/property_feasibility.xlsx
@@ -1723,7 +1723,7 @@
     </row>
     <row r="37" ht="16.5" customHeight="1"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="EE63"/>
   <mergeCells count="30">
     <mergeCell ref="D20:E20"/>
     <mergeCell ref="G10:I10"/>
@@ -2520,7 +2520,7 @@
     </row>
     <row r="37" ht="16.5" customHeight="1"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="EE63"/>
   <mergeCells count="30">
     <mergeCell ref="D20:E20"/>
     <mergeCell ref="G10:I10"/>

</xml_diff>